<commit_message>
feat(documents): review vendor offers with shared spreadsheet components
</commit_message>
<xml_diff>
--- a/public/files/Penawaran-Borneo.xlsx
+++ b/public/files/Penawaran-Borneo.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Harga" sheetId="1" r:id="R0b5755c9243646d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Harga" sheetId="1" r:id="R125d03a642834102"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rincian Penawaran" sheetId="2" r:id="R6f9ad7a096b14734"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,10 +14,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="&quot;Rp &quot;#,##0"/>
+    <x:numFmt numFmtId="201" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -38,8 +40,23 @@
       <x:color rgb="FF1E293B"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:u val="single"/>
+      <x:sz val="11"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -56,8 +73,28 @@
         <x:fgColor rgb="FFE8F1F8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF99DFF3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD1D1D1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFF00"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC1EFCB"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="3">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -73,11 +110,25 @@
         <x:color rgb="FFE2E8F0"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="dotted">
+        <x:color rgb="FF647269"/>
+      </x:left>
+      <x:right style="dotted">
+        <x:color rgb="FF647269"/>
+      </x:right>
+      <x:top style="dotted">
+        <x:color rgb="FF647269"/>
+      </x:top>
+      <x:bottom style="dotted">
+        <x:color rgb="FF647269"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -88,6 +139,24 @@
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="4" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="4" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -413,4 +482,519 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="8" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="8" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="8" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="8" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="8" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="8" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="8" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="12" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="22" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="13" t="str">
+        <x:v>NO.</x:v>
+      </x:c>
+      <x:c r="B9" s="13" t="str">
+        <x:v>URAIAN PEKERJAAN</x:v>
+      </x:c>
+      <x:c r="C9" s="13"/>
+      <x:c r="D9" s="13"/>
+      <x:c r="E9" s="13"/>
+      <x:c r="F9" s="13"/>
+      <x:c r="G9" s="13"/>
+      <x:c r="H9" s="13"/>
+      <x:c r="I9" s="13"/>
+      <x:c r="J9" s="13"/>
+      <x:c r="K9" s="13"/>
+      <x:c r="L9" s="13" t="str">
+        <x:v>VOLUME</x:v>
+      </x:c>
+      <x:c r="M9" s="13"/>
+      <x:c r="N9" s="13" t="str">
+        <x:v>HARGA SATUAN</x:v>
+      </x:c>
+      <x:c r="O9" s="13"/>
+      <x:c r="P9" s="13" t="str">
+        <x:v>JUMLAH HARGA</x:v>
+      </x:c>
+      <x:c r="Q9" s="13"/>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="13"/>
+      <x:c r="B10" s="13"/>
+      <x:c r="C10" s="13"/>
+      <x:c r="D10" s="13"/>
+      <x:c r="E10" s="13"/>
+      <x:c r="F10" s="13"/>
+      <x:c r="G10" s="13"/>
+      <x:c r="H10" s="13"/>
+      <x:c r="I10" s="13"/>
+      <x:c r="J10" s="13"/>
+      <x:c r="K10" s="13"/>
+      <x:c r="L10" s="13"/>
+      <x:c r="M10" s="13"/>
+      <x:c r="N10" s="13" t="str">
+        <x:v>MATERIAL</x:v>
+      </x:c>
+      <x:c r="O10" s="13" t="str">
+        <x:v>JASA</x:v>
+      </x:c>
+      <x:c r="P10" s="13" t="str">
+        <x:v>MATERIAL</x:v>
+      </x:c>
+      <x:c r="Q10" s="13" t="str">
+        <x:v>JASA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="17" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="B11" s="18" t="str">
+        <x:v>Pekerjaan Persiapan</x:v>
+      </x:c>
+      <x:c r="C11" s="17"/>
+      <x:c r="D11" s="15"/>
+      <x:c r="E11" s="15"/>
+      <x:c r="F11" s="15"/>
+      <x:c r="G11" s="15"/>
+      <x:c r="H11" s="15"/>
+      <x:c r="I11" s="15"/>
+      <x:c r="J11" s="15"/>
+      <x:c r="K11" s="15"/>
+      <x:c r="L11" s="15"/>
+      <x:c r="M11" s="15"/>
+      <x:c r="N11" s="15"/>
+      <x:c r="O11" s="15"/>
+      <x:c r="P11" s="16"/>
+      <x:c r="Q11" s="16"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="19" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="B12" s="19" t="str">
+        <x:v>Mobilisasi dan demobilisasi</x:v>
+      </x:c>
+      <x:c r="C12" s="19"/>
+      <x:c r="D12" s="11"/>
+      <x:c r="E12" s="11"/>
+      <x:c r="F12" s="11"/>
+      <x:c r="G12" s="11"/>
+      <x:c r="H12" s="11"/>
+      <x:c r="I12" s="11"/>
+      <x:c r="J12" s="11"/>
+      <x:c r="K12" s="11"/>
+      <x:c r="L12" s="11"/>
+      <x:c r="M12" s="11"/>
+      <x:c r="N12" s="11"/>
+      <x:c r="O12" s="11"/>
+      <x:c r="P12" s="14"/>
+      <x:c r="Q12" s="14" t="n">
+        <x:v>55000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="19" t="str">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="B13" s="19" t="str">
+        <x:v>Pengadaan pipa baja 4 inci</x:v>
+      </x:c>
+      <x:c r="C13" s="19"/>
+      <x:c r="D13" s="11"/>
+      <x:c r="E13" s="11"/>
+      <x:c r="F13" s="11"/>
+      <x:c r="G13" s="11"/>
+      <x:c r="H13" s="11"/>
+      <x:c r="I13" s="11"/>
+      <x:c r="J13" s="11"/>
+      <x:c r="K13" s="11"/>
+      <x:c r="L13" s="11"/>
+      <x:c r="M13" s="11"/>
+      <x:c r="N13" s="11"/>
+      <x:c r="O13" s="11"/>
+      <x:c r="P13" s="14" t="n">
+        <x:v>250000</x:v>
+      </x:c>
+      <x:c r="Q13" s="14"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="11"/>
+      <x:c r="B14" s="11" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="C14" s="11" t="str">
+        <x:v>Pipa termasuk sambungan dan perlindungan selama pengiriman.</x:v>
+      </x:c>
+      <x:c r="D14" s="11"/>
+      <x:c r="E14" s="11"/>
+      <x:c r="F14" s="11"/>
+      <x:c r="G14" s="11"/>
+      <x:c r="H14" s="11"/>
+      <x:c r="I14" s="11"/>
+      <x:c r="J14" s="11"/>
+      <x:c r="K14" s="11"/>
+      <x:c r="L14" s="11"/>
+      <x:c r="M14" s="11"/>
+      <x:c r="N14" s="11"/>
+      <x:c r="O14" s="11"/>
+      <x:c r="P14" s="14"/>
+      <x:c r="Q14" s="14"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="11"/>
+      <x:c r="B15" s="11" t="str">
+        <x:v>1.2.1</x:v>
+      </x:c>
+      <x:c r="C15" s="11" t="str">
+        <x:v>Pemeriksaan spesifikasi material</x:v>
+      </x:c>
+      <x:c r="D15" s="11"/>
+      <x:c r="E15" s="11"/>
+      <x:c r="F15" s="11"/>
+      <x:c r="G15" s="11"/>
+      <x:c r="H15" s="11"/>
+      <x:c r="I15" s="11"/>
+      <x:c r="J15" s="11"/>
+      <x:c r="K15" s="11"/>
+      <x:c r="L15" s="11"/>
+      <x:c r="M15" s="11"/>
+      <x:c r="N15" s="11"/>
+      <x:c r="O15" s="11"/>
+      <x:c r="P15" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q15" s="14"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="19" t="str">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="B16" s="19" t="str">
+        <x:v>Pemasangan pipa</x:v>
+      </x:c>
+      <x:c r="C16" s="19"/>
+      <x:c r="D16" s="11"/>
+      <x:c r="E16" s="11"/>
+      <x:c r="F16" s="11"/>
+      <x:c r="G16" s="11"/>
+      <x:c r="H16" s="11"/>
+      <x:c r="I16" s="11"/>
+      <x:c r="J16" s="11"/>
+      <x:c r="K16" s="11"/>
+      <x:c r="L16" s="11"/>
+      <x:c r="M16" s="11"/>
+      <x:c r="N16" s="11"/>
+      <x:c r="O16" s="11"/>
+      <x:c r="P16" s="14"/>
+      <x:c r="Q16" s="14" t="n">
+        <x:v>110000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="11"/>
+      <x:c r="B17" s="11" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="C17" s="11" t="str">
+        <x:v>Persiapan area dan pemeriksaan sambungan.</x:v>
+      </x:c>
+      <x:c r="D17" s="11"/>
+      <x:c r="E17" s="11"/>
+      <x:c r="F17" s="11"/>
+      <x:c r="G17" s="11"/>
+      <x:c r="H17" s="11"/>
+      <x:c r="I17" s="11"/>
+      <x:c r="J17" s="11"/>
+      <x:c r="K17" s="11"/>
+      <x:c r="L17" s="11"/>
+      <x:c r="M17" s="11"/>
+      <x:c r="N17" s="11"/>
+      <x:c r="O17" s="11"/>
+      <x:c r="P17" s="14"/>
+      <x:c r="Q17" s="14"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="19" t="str">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="B18" s="19" t="str">
+        <x:v>Katup gate 4 inci</x:v>
+      </x:c>
+      <x:c r="C18" s="19"/>
+      <x:c r="D18" s="11"/>
+      <x:c r="E18" s="11"/>
+      <x:c r="F18" s="11"/>
+      <x:c r="G18" s="11"/>
+      <x:c r="H18" s="11"/>
+      <x:c r="I18" s="11"/>
+      <x:c r="J18" s="11"/>
+      <x:c r="K18" s="11"/>
+      <x:c r="L18" s="11"/>
+      <x:c r="M18" s="11"/>
+      <x:c r="N18" s="11"/>
+      <x:c r="O18" s="11"/>
+      <x:c r="P18" s="14" t="n">
+        <x:v>680000</x:v>
+      </x:c>
+      <x:c r="Q18" s="14"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="11"/>
+      <x:c r="B19" s="11"/>
+      <x:c r="C19" s="11"/>
+      <x:c r="D19" s="11"/>
+      <x:c r="E19" s="11"/>
+      <x:c r="F19" s="11"/>
+      <x:c r="G19" s="11"/>
+      <x:c r="H19" s="11"/>
+      <x:c r="I19" s="11"/>
+      <x:c r="J19" s="11"/>
+      <x:c r="K19" s="11"/>
+      <x:c r="L19" s="11"/>
+      <x:c r="M19" s="11"/>
+      <x:c r="N19" s="11"/>
+      <x:c r="O19" s="11"/>
+      <x:c r="P19" s="14"/>
+      <x:c r="Q19" s="14"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="22"/>
+      <x:c r="B20" s="22" t="str">
+        <x:v>SUBTOTAL</x:v>
+      </x:c>
+      <x:c r="C20" s="22"/>
+      <x:c r="D20" s="20"/>
+      <x:c r="E20" s="20"/>
+      <x:c r="F20" s="20"/>
+      <x:c r="G20" s="20"/>
+      <x:c r="H20" s="20"/>
+      <x:c r="I20" s="20"/>
+      <x:c r="J20" s="20"/>
+      <x:c r="K20" s="20"/>
+      <x:c r="L20" s="20"/>
+      <x:c r="M20" s="20"/>
+      <x:c r="N20" s="20"/>
+      <x:c r="O20" s="20"/>
+      <x:c r="P20" s="23" t="n">
+        <x:v>930000</x:v>
+      </x:c>
+      <x:c r="Q20" s="23" t="n">
+        <x:v>165000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="17" t="str">
+        <x:v>II</x:v>
+      </x:c>
+      <x:c r="B21" s="18" t="str">
+        <x:v>Pekerjaan Finishing</x:v>
+      </x:c>
+      <x:c r="C21" s="17"/>
+      <x:c r="D21" s="15"/>
+      <x:c r="E21" s="15"/>
+      <x:c r="F21" s="15"/>
+      <x:c r="G21" s="15"/>
+      <x:c r="H21" s="15"/>
+      <x:c r="I21" s="15"/>
+      <x:c r="J21" s="15"/>
+      <x:c r="K21" s="15"/>
+      <x:c r="L21" s="15"/>
+      <x:c r="M21" s="15"/>
+      <x:c r="N21" s="15"/>
+      <x:c r="O21" s="15"/>
+      <x:c r="P21" s="16"/>
+      <x:c r="Q21" s="16"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="26" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="B22" s="26" t="str">
+        <x:v>Pengujian dan serah terima</x:v>
+      </x:c>
+      <x:c r="C22" s="26"/>
+      <x:c r="D22" s="24"/>
+      <x:c r="E22" s="24"/>
+      <x:c r="F22" s="24"/>
+      <x:c r="G22" s="24"/>
+      <x:c r="H22" s="24"/>
+      <x:c r="I22" s="24"/>
+      <x:c r="J22" s="24"/>
+      <x:c r="K22" s="24"/>
+      <x:c r="L22" s="24"/>
+      <x:c r="M22" s="24"/>
+      <x:c r="N22" s="24"/>
+      <x:c r="O22" s="24"/>
+      <x:c r="P22" s="25"/>
+      <x:c r="Q22" s="25"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="19" t="str">
+        <x:v>2.1</x:v>
+      </x:c>
+      <x:c r="B23" s="19" t="str">
+        <x:v>Pengujian sambungan</x:v>
+      </x:c>
+      <x:c r="C23" s="19"/>
+      <x:c r="D23" s="11"/>
+      <x:c r="E23" s="11"/>
+      <x:c r="F23" s="11"/>
+      <x:c r="G23" s="11"/>
+      <x:c r="H23" s="11"/>
+      <x:c r="I23" s="11"/>
+      <x:c r="J23" s="11"/>
+      <x:c r="K23" s="11"/>
+      <x:c r="L23" s="11"/>
+      <x:c r="M23" s="11"/>
+      <x:c r="N23" s="11"/>
+      <x:c r="O23" s="11"/>
+      <x:c r="P23" s="14"/>
+      <x:c r="Q23" s="14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="22"/>
+      <x:c r="B24" s="22" t="str">
+        <x:v>SUBTOTAL</x:v>
+      </x:c>
+      <x:c r="C24" s="22"/>
+      <x:c r="D24" s="20"/>
+      <x:c r="E24" s="20"/>
+      <x:c r="F24" s="20"/>
+      <x:c r="G24" s="20"/>
+      <x:c r="H24" s="20"/>
+      <x:c r="I24" s="20"/>
+      <x:c r="J24" s="20"/>
+      <x:c r="K24" s="20"/>
+      <x:c r="L24" s="20"/>
+      <x:c r="M24" s="20"/>
+      <x:c r="N24" s="20"/>
+      <x:c r="O24" s="20"/>
+      <x:c r="P24" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q24" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="19"/>
+      <x:c r="B25" s="19" t="str">
+        <x:v>TOTAL SUB JUMLAH I-II</x:v>
+      </x:c>
+      <x:c r="C25" s="19"/>
+      <x:c r="D25" s="11"/>
+      <x:c r="E25" s="11"/>
+      <x:c r="F25" s="11"/>
+      <x:c r="G25" s="11"/>
+      <x:c r="H25" s="11"/>
+      <x:c r="I25" s="11"/>
+      <x:c r="J25" s="11"/>
+      <x:c r="K25" s="11"/>
+      <x:c r="L25" s="11"/>
+      <x:c r="M25" s="11"/>
+      <x:c r="N25" s="11"/>
+      <x:c r="O25" s="11"/>
+      <x:c r="P25" s="27" t="n">
+        <x:v>930000</x:v>
+      </x:c>
+      <x:c r="Q25" s="27" t="n">
+        <x:v>165000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="19"/>
+      <x:c r="B26" s="19" t="str">
+        <x:v>TOTAL SUB JUMLAH</x:v>
+      </x:c>
+      <x:c r="C26" s="19"/>
+      <x:c r="D26" s="11"/>
+      <x:c r="E26" s="11"/>
+      <x:c r="F26" s="11"/>
+      <x:c r="G26" s="11"/>
+      <x:c r="H26" s="11"/>
+      <x:c r="I26" s="11"/>
+      <x:c r="J26" s="11"/>
+      <x:c r="K26" s="11"/>
+      <x:c r="L26" s="11"/>
+      <x:c r="M26" s="11"/>
+      <x:c r="N26" s="11"/>
+      <x:c r="O26" s="11"/>
+      <x:c r="P26" s="27"/>
+      <x:c r="Q26" s="27" t="n">
+        <x:v>1095000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="19"/>
+      <x:c r="B27" s="19" t="str">
+        <x:v>TERBILANG: SATU JUTA SEMBILAN PULUH LIMA RIBU RUPIAH</x:v>
+      </x:c>
+      <x:c r="C27" s="19"/>
+      <x:c r="D27" s="11"/>
+      <x:c r="E27" s="11"/>
+      <x:c r="F27" s="11"/>
+      <x:c r="G27" s="11"/>
+      <x:c r="H27" s="11"/>
+      <x:c r="I27" s="11"/>
+      <x:c r="J27" s="11"/>
+      <x:c r="K27" s="11"/>
+      <x:c r="L27" s="11"/>
+      <x:c r="M27" s="11"/>
+      <x:c r="N27" s="11"/>
+      <x:c r="O27" s="11"/>
+      <x:c r="P27" s="27"/>
+      <x:c r="Q27" s="27"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="11"/>
+      <x:c r="B28" s="11"/>
+      <x:c r="C28" s="11"/>
+      <x:c r="D28" s="11"/>
+      <x:c r="E28" s="11"/>
+      <x:c r="F28" s="11"/>
+      <x:c r="G28" s="11"/>
+      <x:c r="H28" s="11"/>
+      <x:c r="I28" s="11"/>
+      <x:c r="J28" s="11"/>
+      <x:c r="K28" s="11"/>
+      <x:c r="L28" s="11" t="str">
+        <x:v>Dibuat oleh</x:v>
+      </x:c>
+      <x:c r="M28" s="11"/>
+      <x:c r="N28" s="11"/>
+      <x:c r="O28" s="11"/>
+      <x:c r="P28" s="11"/>
+      <x:c r="Q28" s="11"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A9:A10"/>
+    <x:mergeCell ref="B9:K10"/>
+    <x:mergeCell ref="L9:M10"/>
+    <x:mergeCell ref="N9:O9"/>
+    <x:mergeCell ref="P9:Q9"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>